<commit_message>
Apply provisional student identity formats and dropdowns
</commit_message>
<xml_diff>
--- a/apps/web/public/templates/students-temp.xlsx
+++ b/apps/web/public/templates/students-temp.xlsx
@@ -146,6 +146,31 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>OpenAI</author>
+  </authors>
+  <commentList>
+    <comment ref="F1" authorId="0" shapeId="0">
+      <text>
+        <t>القائمة مؤقتة بانتظار اعتماد الجامعة.</t>
+      </text>
+    </comment>
+    <comment ref="H1" authorId="0" shapeId="0">
+      <text>
+        <t>القائمة مؤقتة بانتظار اعتماد الجامعة.</t>
+      </text>
+    </comment>
+    <comment ref="X1" authorId="0" shapeId="0">
+      <text>
+        <t>القائمة مؤقتة بانتظار اعتماد الجامعة.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3991,7 +4016,19 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:X500"/>
+  <dataValidations count="3">
+    <dataValidation sqref="F2:F1001" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="قائمة مقترحة مؤقتة" prompt="اختر الجنس من القائمة." type="list">
+      <formula1>"ذكر,أنثى"</formula1>
+    </dataValidation>
+    <dataValidation sqref="H2:H1001" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="قائمة مقترحة مؤقتة" prompt="اختر الجنسية من القائمة أو اختر أخرى." type="list">
+      <formula1>"سوري,تركي,فلسطيني,أردني,لبناني,عراقي,مصري,سعودي,يمني,إماراتي,قطري,كويتي,عُماني,بحريني,أخرى"</formula1>
+    </dataValidation>
+    <dataValidation sqref="X2:X1001" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="قائمة مقترحة مؤقتة" prompt="اختر مكان الولادة من القائمة أو اختر مكانًا آخر." type="list">
+      <formula1>"دمشق,ريف دمشق,حلب,حمص,حماة,اللاذقية,طرطوس,إدلب,درعا,السويداء,القنيطرة,دير الزور,الرقة,الحسكة,خارج سوريا / مكان آخر"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 
@@ -4025,7 +4062,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>الرقم الجامعي، الاسم الأول، اسم الأب، اسم العائلة، اسم الأم، الرقم الوطني، رقم الاكتتاب، مكان الولادة.</t>
+          <t>الحقول الإلزامية: الرقم الجامعي، الأسماء، اسم الأم، الرقم الوطني (11 رقمًا مؤقتًا)، رقم الاكتتاب، ومكان الولادة.</t>
         </is>
       </c>
     </row>
@@ -4061,7 +4098,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>استخدم تاريخًا بصيغة 2026-09-01.</t>
+          <t>التواريخ: استخدم تاريخًا بصيغة 2026-09-01. الهاتف السوري المحلي، إن أُدخل، 10 أرقام ويبدأ بـ 09.</t>
         </is>
       </c>
     </row>
@@ -4073,7 +4110,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>يجب أن تطابق بيانات التحقق سجل الجامعة، ويُرفض الصف الناقص أو المكرر قبل الاستيراد.</t>
+          <t>تطابق البيانات: يجب أن تطابق بيانات التحقق سجل الجامعة. تُرفض الأسماء غير الصالحة والأرقام المخالفة أو المكررة قبل الاستيراد.</t>
         </is>
       </c>
     </row>
@@ -4085,11 +4122,17 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>بعد الاستيراد، ينشئ الطالب حسابه بهذه البيانات ثم يعيّن كلمة المرور.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="28" customHeight="1"/>
+          <t>إنشاء الحساب: بعد الاستيراد، ينشئ الطالب حسابه بهذه البيانات ثم يعيّن كلمة المرور.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="28" customHeight="1">
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>ملاحظة مؤقتة: صيغة الرقم الوطني والهاتف وقوائم الجنسية ومكان الولادة بانتظار اعتماد الجامعة.</t>
+        </is>
+      </c>
+    </row>
     <row r="10" ht="28" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>

</xml_diff>